<commit_message>
feat: modularize core trading and fund management logic into separate source files and initialize error logging.
</commit_message>
<xml_diff>
--- a/Master.xlsx
+++ b/Master.xlsx
@@ -1,87 +1,33 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Pr\Work\pr\CFrepo\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="-105" yWindow="-105" windowWidth="23250" windowHeight="12450"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-105" yWindow="-105" windowWidth="23250" windowHeight="12450" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Users" sheetId="1" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Users" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <definedNames/>
+  <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="15">
-  <si>
-    <t>uci</t>
-  </si>
-  <si>
-    <t>first_name</t>
-  </si>
-  <si>
-    <t>last_name</t>
-  </si>
-  <si>
-    <t>mobile</t>
-  </si>
-  <si>
-    <t>communication email</t>
-  </si>
-  <si>
-    <t>account_email</t>
-  </si>
-  <si>
-    <t>intraday</t>
-  </si>
-  <si>
-    <t>zerodha_access_token</t>
-  </si>
-  <si>
-    <t>current_value</t>
-  </si>
-  <si>
-    <t>bank_fund</t>
-  </si>
-  <si>
-    <t>ipo_blocked_fund</t>
-  </si>
-  <si>
-    <t>holdings_total_value</t>
-  </si>
-  <si>
-    <t>broker_withdrawable_fund</t>
-  </si>
-  <si>
-    <t>broker_investable_fund</t>
-  </si>
-  <si>
-    <t>still_needed_amount</t>
-  </si>
-</sst>
-</file>
-
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="1" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="0"/>
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <color theme="1"/>
+      <sz val="11"/>
       <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -100,24 +46,83 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="2">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
@@ -417,86 +422,166 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:AE3"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col min="9" max="9" width="11.85546875" customWidth="1"/>
-    <col min="10" max="10" width="10.28515625" customWidth="1"/>
-    <col min="11" max="11" width="16.28515625" customWidth="1"/>
+    <col width="11.85546875" customWidth="1" min="9" max="9"/>
+    <col width="10.28515625" customWidth="1" min="10" max="10"/>
+    <col width="16.28515625" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:31" ht="43.15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
+    <row r="1" ht="43.15" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>uci</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>first_name</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>last_name</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>mobile</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>communication email</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>account_email</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>intraday</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>zerodha_access_token</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>current_value</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>bank_fund</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>ipo_blocked_fund</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>holdings_total_value</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>broker_withdrawable_fund</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>broker_investable_fund</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>still_needed_amount</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="n"/>
+      <c r="Q1" s="1" t="n"/>
+      <c r="R1" s="1" t="n"/>
+      <c r="S1" s="1" t="n"/>
+      <c r="T1" s="1" t="n"/>
+      <c r="U1" s="1" t="n"/>
+      <c r="V1" s="1" t="n"/>
+      <c r="W1" s="1" t="n"/>
+      <c r="X1" s="1" t="n"/>
+      <c r="Y1" s="1" t="n"/>
+      <c r="Z1" s="1" t="n"/>
+      <c r="AA1" s="1" t="n"/>
+      <c r="AB1" s="1" t="n"/>
+      <c r="AC1" s="1" t="n"/>
+      <c r="AD1" s="1" t="n"/>
+      <c r="AE1" s="1" t="n"/>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Prakhar</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>prakharvasishtha9@gmail.com</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>tok_123</t>
+        </is>
+      </c>
+      <c r="I2" t="n">
+        <v>250000</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="J1" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="K1" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="L1" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="M1" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="N1" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="O1" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="P1" s="1"/>
-      <c r="Q1" s="1"/>
-      <c r="R1" s="1"/>
-      <c r="S1" s="1"/>
-      <c r="T1" s="1"/>
-      <c r="U1" s="1"/>
-      <c r="V1" s="1"/>
-      <c r="W1" s="1"/>
-      <c r="X1" s="1"/>
-      <c r="Y1" s="1"/>
-      <c r="Z1" s="1"/>
-      <c r="AA1" s="1"/>
-      <c r="AB1" s="1"/>
-      <c r="AC1" s="1"/>
-      <c r="AD1" s="1"/>
-      <c r="AE1" s="1"/>
-    </row>
-    <row r="2" spans="1:31" x14ac:dyDescent="0.25">
-      <c r="A2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3" spans="1:31" x14ac:dyDescent="0.25">
-      <c r="A3">
-        <v>2</v>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Sonam</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>sonampvasishtha@gmail.com</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>tok_456</t>
+        </is>
+      </c>
+      <c r="I3" t="n">
+        <v>180000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>